<commit_message>
Apply full-text verification of 8 open-access studies
Verified against open-access full texts: R242, R269, R088, O15 (core)
and R081, R093, R102, R129. Changes: Q7 for 7 studies, Z (R088, R093),
T (R093, R102, R269), q5 (R102, R129), q4 (R129). The other 72 studies
stay abstract-based; fulltext_verified.json gives the reason for each.

Updates final.json, extraction.txt, the Excel workbook and Appendix B.
make_appB.py now keeps CRLF line endings.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XqnX2YwxoAxecfihx1cP3d
</commit_message>
<xml_diff>
--- a/thesis-repo/review_data/SLR_Search_and_Screening.xlsx
+++ b/thesis-repo/review_data/SLR_Search_and_Screening.xlsx
@@ -23157,14 +23157,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="inlineStr">
         <is>
           <t>trust_ethics</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -23333,7 +23330,6 @@
           <t>p2: na -&gt; +</t>
         </is>
       </c>
-      <c r="AK3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -23487,14 +23483,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr">
         <is>
           <t>dynamism</t>
         </is>
       </c>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -23648,7 +23641,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH5" t="inlineStr"/>
       <c r="AI5" t="inlineStr">
         <is>
           <t>platform, data_infra</t>
@@ -23659,7 +23651,6 @@
           <t>design: Qualitative/case -&gt; Mixed</t>
         </is>
       </c>
-      <c r="AK5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -23813,7 +23804,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH6" t="inlineStr"/>
       <c r="AI6" t="inlineStr">
         <is>
           <t>data_infra, resources</t>
@@ -23824,7 +23814,6 @@
           <t>p2: + -&gt; na; s: True -&gt; False; z: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -23978,14 +23967,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr">
         <is>
           <t>trust_ethics</t>
         </is>
       </c>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -24139,7 +24125,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="inlineStr">
         <is>
           <t>dynamism, data_infra, resources</t>
@@ -24150,7 +24135,6 @@
           <t>s: False -&gt; True; q2: 1 -&gt; 0; q4: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -24304,7 +24288,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="inlineStr">
         <is>
           <t>integration</t>
@@ -24315,7 +24298,6 @@
           <t>z: False -&gt; True; q2: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -24469,7 +24451,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH10" t="inlineStr"/>
       <c r="AI10" t="inlineStr">
         <is>
           <t>integration</t>
@@ -24480,7 +24461,6 @@
           <t>design: Survey -&gt; Mixed; p1: + -&gt; na; z: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -24634,14 +24614,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH11" t="inlineStr"/>
       <c r="AI11" t="inlineStr">
         <is>
           <t>dynamism, resources</t>
         </is>
       </c>
-      <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -24795,7 +24772,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH12" t="inlineStr"/>
       <c r="AI12" t="inlineStr">
         <is>
           <t>integration</t>
@@ -24806,7 +24782,6 @@
           <t>outcome: FP -&gt; INNOV; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -24960,14 +24935,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
       <c r="AJ13" t="inlineStr">
         <is>
           <t>p2: + -&gt; 0; q2: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -25121,7 +25093,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH14" t="inlineStr"/>
       <c r="AI14" t="inlineStr">
         <is>
           <t>integration, dynamism, trust_ethics</t>
@@ -25132,7 +25103,6 @@
           <t>p2: + -&gt; na; q3: 0 -&gt; 1; q4: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -25286,7 +25256,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH15" t="inlineStr"/>
       <c r="AI15" t="inlineStr">
         <is>
           <t>cognition, data_infra</t>
@@ -25297,7 +25266,6 @@
           <t>s: False -&gt; True; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -25461,7 +25429,6 @@
           <t>s: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -25615,14 +25582,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH17" t="inlineStr"/>
       <c r="AI17" t="inlineStr">
         <is>
           <t>cognition, integration</t>
         </is>
       </c>
-      <c r="AJ17" t="inlineStr"/>
-      <c r="AK17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -25776,7 +25740,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH18" t="inlineStr"/>
       <c r="AI18" t="inlineStr">
         <is>
           <t>data_infra</t>
@@ -25787,7 +25750,6 @@
           <t>s: True -&gt; False; t: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -25941,7 +25903,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH19" t="inlineStr"/>
       <c r="AI19" t="inlineStr">
         <is>
           <t>integration</t>
@@ -25952,7 +25913,6 @@
           <t>t: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -26106,7 +26066,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH20" t="inlineStr"/>
       <c r="AI20" t="inlineStr">
         <is>
           <t>dynamism</t>
@@ -26117,7 +26076,6 @@
           <t>design: Panel/archival -&gt; Survey; q6: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -26271,7 +26229,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH21" t="inlineStr"/>
       <c r="AI21" t="inlineStr">
         <is>
           <t>cognition, resources</t>
@@ -26282,7 +26239,6 @@
           <t>outcome: FP -&gt; INNOV; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -26609,7 +26565,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH23" t="inlineStr"/>
       <c r="AI23" t="inlineStr">
         <is>
           <t>trust_ethics, data_infra, platform</t>
@@ -26620,7 +26575,6 @@
           <t>p1: + -&gt; na; s: True -&gt; False; q2: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -26774,7 +26728,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH24" t="inlineStr"/>
       <c r="AI24" t="inlineStr">
         <is>
           <t>resources, cognition</t>
@@ -26785,7 +26738,6 @@
           <t>q4: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -26954,7 +26906,6 @@
           <t>outcome: RES -&gt; INNOV; p1: na -&gt; +; t: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -27108,14 +27059,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH26" t="inlineStr"/>
       <c r="AI26" t="inlineStr">
         <is>
           <t>data_infra, dynamism</t>
         </is>
       </c>
-      <c r="AJ26" t="inlineStr"/>
-      <c r="AK26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -27279,8 +27227,6 @@
           <t>dynamism</t>
         </is>
       </c>
-      <c r="AJ27" t="inlineStr"/>
-      <c r="AK27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -27434,7 +27380,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH28" t="inlineStr"/>
       <c r="AI28" t="inlineStr">
         <is>
           <t>dynamism</t>
@@ -27445,7 +27390,6 @@
           <t>design: Survey -&gt; Mixed; s: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -27599,7 +27543,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH29" t="inlineStr"/>
       <c r="AI29" t="inlineStr">
         <is>
           <t>resources, integration, trust_ethics</t>
@@ -27610,7 +27553,6 @@
           <t>p1: na -&gt; +; q4: 1 -&gt; 0; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -27952,7 +27894,6 @@
           <t>q4: 1 -&gt; 0; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -28121,7 +28062,6 @@
           <t>s: True -&gt; False; t: True -&gt; False; q4: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -28275,7 +28215,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH33" t="inlineStr"/>
       <c r="AI33" t="inlineStr">
         <is>
           <t>integration, data_infra</t>
@@ -28286,7 +28225,6 @@
           <t>q2: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -28440,7 +28378,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH34" t="inlineStr"/>
       <c r="AI34" t="inlineStr">
         <is>
           <t>resources, integration</t>
@@ -28451,7 +28388,6 @@
           <t>outcome: FP -&gt; CA</t>
         </is>
       </c>
-      <c r="AK34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -28620,7 +28556,6 @@
           <t>q4: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -28784,8 +28719,6 @@
           <t>integration</t>
         </is>
       </c>
-      <c r="AJ36" t="inlineStr"/>
-      <c r="AK36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -28895,7 +28828,7 @@
       </c>
       <c r="V37" s="2" t="inlineStr">
         <is>
-          <t>Abstract only; limitations not assessable unless stated in abstract</t>
+          <t>Section 8 'Limitations and Research Agenda' (AAM p. 22): cross-sectional design, Delhi NCR only</t>
         </is>
       </c>
       <c r="W37" s="2" t="n">
@@ -28936,17 +28869,24 @@
       </c>
       <c r="AG37" t="inlineStr">
         <is>
-          <t>Abstract-based</t>
-        </is>
-      </c>
-      <c r="AH37" t="inlineStr"/>
+          <t>Full text verified</t>
+        </is>
+      </c>
+      <c r="AH37" t="inlineStr">
+        <is>
+          <t>https://eprints.lancs.ac.uk/id/eprint/232040/ (author accepted manuscript)</t>
+        </is>
+      </c>
       <c r="AI37" t="inlineStr">
         <is>
           <t>dynamism</t>
         </is>
       </c>
-      <c r="AJ37" t="inlineStr"/>
-      <c r="AK37" t="inlineStr"/>
+      <c r="AK37" t="inlineStr">
+        <is>
+          <t>Full-text check: abstract coding confirmed. Full text confirms abstract coding. AIC-&gt;exploitation .514, -&gt;exploration .651; effect on export performance indirect via ambidexterity and IMC. H5 (exploitation-&gt;EP) and moderations H9a/H10a not supported; codes unaffected.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -29100,7 +29040,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH38" t="inlineStr"/>
       <c r="AI38" t="inlineStr">
         <is>
           <t>integration</t>
@@ -29111,7 +29050,6 @@
           <t>p2: + -&gt; na</t>
         </is>
       </c>
-      <c r="AK38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -29265,7 +29203,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH39" t="inlineStr"/>
       <c r="AI39" t="inlineStr">
         <is>
           <t>dynamism, data_infra</t>
@@ -29276,7 +29213,6 @@
           <t>s: False -&gt; True; z: False -&gt; True; q2: 0 -&gt; 1; q6: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -29603,7 +29539,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH41" t="inlineStr"/>
       <c r="AI41" t="inlineStr">
         <is>
           <t>integration, imitability</t>
@@ -29614,7 +29549,6 @@
           <t>p2: + -&gt; c; z: True -&gt; False; t: True -&gt; False; q2: 1 -&gt; 0; q4: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -29679,34 +29613,34 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>AI capabilities translated into competitive positioning via orchestration and network effects</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>Orchestration, network effects</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N42" s="2" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="O42" s="2" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="P42" s="2" t="inlineStr">
-        <is>
-          <t>AI capabilities translated into competitive positioning via orchestration and network effects</t>
-        </is>
-      </c>
-      <c r="Q42" s="2" t="inlineStr">
-        <is>
-          <t>Orchestration, network effects</t>
-        </is>
-      </c>
-      <c r="R42" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="S42" s="2" t="inlineStr">
         <is>
           <t>+</t>
@@ -29724,7 +29658,7 @@
       </c>
       <c r="V42" s="2" t="inlineStr">
         <is>
-          <t>Abstract only; limitations not assessable unless stated in abstract</t>
+          <t>No limitations section; only Section 6 'Future Research Directions' (p. 658)</t>
         </is>
       </c>
       <c r="W42" s="2" t="n">
@@ -29747,7 +29681,7 @@
       </c>
       <c r="AC42" s="2" t="inlineStr">
         <is>
-          <t>not assessable</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AD42" s="2" t="n">
@@ -29765,10 +29699,14 @@
       </c>
       <c r="AG42" t="inlineStr">
         <is>
-          <t>Abstract-based</t>
-        </is>
-      </c>
-      <c r="AH42" t="inlineStr"/>
+          <t>Full text verified</t>
+        </is>
+      </c>
+      <c r="AH42" t="inlineStr">
+        <is>
+          <t>https://cspub-ijcisim.org/index.php/ijcisim/article/download/2978/2354 (published version)</t>
+        </is>
+      </c>
       <c r="AI42" t="inlineStr">
         <is>
           <t>platform</t>
@@ -29779,7 +29717,11 @@
           <t>z: True -&gt; False; t: False -&gt; True; q4: 0 -&gt; 1; q5: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK42" t="inlineStr"/>
+      <c r="AK42" t="inlineStr">
+        <is>
+          <t>Full-text check: z: False -&gt; True; q7: not_assessable -&gt; no. Z added: platform ecosystem orchestration as capacity to 'organize and mobilize relationships' to co-create value (pp. 655-656). Outcome kept CA: 'Dynamic Competitive Positioning' is named the primary strategic output (Sec. 3.4); SCA only appears as a downstream proposition (P5). Sections 3.2 and 3.3 repeat the same text.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -29948,7 +29890,6 @@
           <t>z: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -30008,29 +29949,29 @@
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>AI-driven risk management associated with supply chain resilience</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N44" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O44" s="2" t="inlineStr">
-        <is>
-          <t>Resilience</t>
-        </is>
-      </c>
-      <c r="P44" s="2" t="inlineStr">
-        <is>
-          <t>AI-driven risk management associated with supply chain resilience</t>
-        </is>
-      </c>
-      <c r="Q44" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="R44" s="2" t="inlineStr">
         <is>
           <t>Supply chain complexity</t>
@@ -30053,7 +29994,7 @@
       </c>
       <c r="V44" s="2" t="inlineStr">
         <is>
-          <t>Abstract only; limitations not assessable unless stated in abstract</t>
+          <t>Discussion, p. 215: five limitations (cross-sectional, single country, single respondent, parsimonious model, no sustainability outcome)</t>
         </is>
       </c>
       <c r="W44" s="2" t="n">
@@ -30094,17 +30035,24 @@
       </c>
       <c r="AG44" t="inlineStr">
         <is>
-          <t>Abstract-based</t>
-        </is>
-      </c>
-      <c r="AH44" t="inlineStr"/>
+          <t>Full text verified</t>
+        </is>
+      </c>
+      <c r="AH44" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.33168/JLISS.2026.1010 (published version, open access)</t>
+        </is>
+      </c>
       <c r="AI44" t="inlineStr">
         <is>
           <t>dynamism, data_infra</t>
         </is>
       </c>
-      <c r="AJ44" t="inlineStr"/>
-      <c r="AK44" t="inlineStr"/>
+      <c r="AK44" t="inlineStr">
+        <is>
+          <t>Full-text check: z: False -&gt; True; t: False -&gt; True. Z and T added: AI strengthens sensing, seizing (decision support, rapid resource reallocation) and reconfiguring (real-time optimisation) (p. 204; Discussion p. 213). Direct effect small (beta=.102).</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -30258,7 +30206,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH45" t="inlineStr"/>
       <c r="AI45" t="inlineStr">
         <is>
           <t>dynamism</t>
@@ -30269,7 +30216,6 @@
           <t>p1: + -&gt; na; z: True -&gt; False; t: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -30423,7 +30369,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH46" t="inlineStr"/>
       <c r="AI46" t="inlineStr">
         <is>
           <t>integration, dynamism, data_infra, cognition</t>
@@ -30434,7 +30379,6 @@
           <t>s: False -&gt; True; q4: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -30504,7 +30448,7 @@
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>x</t>
         </is>
       </c>
       <c r="O47" s="2" t="inlineStr">
@@ -30544,7 +30488,7 @@
       </c>
       <c r="V47" s="2" t="inlineStr">
         <is>
-          <t>Abstract only; limitations not assessable unless stated in abstract</t>
+          <t>Section 5.3 'Limitations and further research directions' (AAM p. 21): generalisability, cross-sectional design</t>
         </is>
       </c>
       <c r="W47" s="2" t="n">
@@ -30560,18 +30504,18 @@
         <v>1</v>
       </c>
       <c r="AA47" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB47" s="2" t="n">
         <v>1</v>
       </c>
       <c r="AC47" s="2" t="inlineStr">
         <is>
-          <t>not assessable</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AD47" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE47" t="inlineStr">
         <is>
@@ -30580,15 +30524,19 @@
       </c>
       <c r="AF47" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="AG47" t="inlineStr">
         <is>
-          <t>Abstract-based</t>
-        </is>
-      </c>
-      <c r="AH47" t="inlineStr"/>
+          <t>Full text verified</t>
+        </is>
+      </c>
+      <c r="AH47" t="inlineStr">
+        <is>
+          <t>https://researchonline.ljmu.ac.uk/id/eprint/11948/ (author accepted manuscript)</t>
+        </is>
+      </c>
       <c r="AI47" t="inlineStr">
         <is>
           <t>cognition, dynamism</t>
@@ -30599,7 +30547,11 @@
           <t>p2: na -&gt; +; s: False -&gt; True; z: False -&gt; True; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK47" t="inlineStr"/>
+      <c r="AK47" t="inlineStr">
+        <is>
+          <t>Full-text check: t: False -&gt; True; q5: 0 -&gt; 1; q7: not_assessable -&gt; yes. BDA-AI-&gt;OP beta=.52 (Table 4). T added: BDA-AI insights 'create opportunities for organisations to reconfigure their resources' (AAM p. 10, H3). q5 0-&gt;1: PLS-SEM with bootstrapping, reliability/validity tests, endogeneity check (NLBCDR).</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -30768,7 +30720,6 @@
           <t>z: False -&gt; True; q2: 0 -&gt; 1; q6: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -30937,7 +30888,6 @@
           <t>s: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -31106,7 +31056,6 @@
           <t>t: True -&gt; False; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -31260,14 +31209,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH51" t="inlineStr"/>
       <c r="AI51" t="inlineStr">
         <is>
           <t>data_infra, integration</t>
         </is>
       </c>
-      <c r="AJ51" t="inlineStr"/>
-      <c r="AK51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -31436,7 +31382,6 @@
           <t>p2: na -&gt; +</t>
         </is>
       </c>
-      <c r="AK52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -31590,7 +31535,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH53" t="inlineStr"/>
       <c r="AI53" t="inlineStr">
         <is>
           <t>data_infra, integration, trust_ethics, dynamism, imitability</t>
@@ -31601,7 +31545,6 @@
           <t>z: False -&gt; True; q4: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -31770,7 +31713,6 @@
           <t>q6: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -31924,7 +31866,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH55" t="inlineStr"/>
       <c r="AI55" t="inlineStr">
         <is>
           <t>integration</t>
@@ -31935,7 +31876,6 @@
           <t>t: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -32104,7 +32044,6 @@
           <t>s: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -32258,7 +32197,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH57" t="inlineStr"/>
       <c r="AI57" t="inlineStr">
         <is>
           <t>integration</t>
@@ -32269,7 +32207,6 @@
           <t>outcome: FP -&gt; INNOV; p2: na -&gt; +; z: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -32379,7 +32316,7 @@
       </c>
       <c r="V58" s="2" t="inlineStr">
         <is>
-          <t>Abstract only; limitations not assessable unless stated in abstract</t>
+          <t>No limitations section for the empirical studies; only a robustness note on writing quality (p. 13) and limits of AI itself (Sec. 5.2)</t>
         </is>
       </c>
       <c r="W58" s="2" t="n">
@@ -32392,21 +32329,21 @@
         <v>1</v>
       </c>
       <c r="Z58" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA58" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB58" s="2" t="n">
         <v>1</v>
       </c>
       <c r="AC58" s="2" t="inlineStr">
         <is>
-          <t>not assessable</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AD58" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AE58" t="inlineStr">
         <is>
@@ -32415,15 +32352,19 @@
       </c>
       <c r="AF58" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="AG58" t="inlineStr">
         <is>
-          <t>Abstract-based</t>
-        </is>
-      </c>
-      <c r="AH58" t="inlineStr"/>
+          <t>Full text verified</t>
+        </is>
+      </c>
+      <c r="AH58" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2408.08811 (preprint v1, 16 Aug 2024; may differ from the Strategy Science version)</t>
+        </is>
+      </c>
       <c r="AI58" t="inlineStr">
         <is>
           <t>dynamism, imitability, cognition</t>
@@ -32434,7 +32375,11 @@
           <t>design: Conceptual -&gt; Mixed; p2: + -&gt; na; q4: 1 -&gt; 0; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK58" t="inlineStr"/>
+      <c r="AK58" t="inlineStr">
+        <is>
+          <t>Full-text check: q4: 0 -&gt; 1; q5: 0 -&gt; 1; q7: not_assessable -&gt; no. P1 c confirmed: effect on firm performance 'depends on competitive dynamics' (Sec. 5.1). q4 0-&gt;1 (samples fully described), q5 0-&gt;1 (pre-registered experiment, regressions with robust SEs, ICC).</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -32603,7 +32548,6 @@
           <t>p2: + -&gt; na; t: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -32757,7 +32701,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH60" t="inlineStr"/>
       <c r="AI60" t="inlineStr">
         <is>
           <t>cognition</t>
@@ -32768,7 +32711,6 @@
           <t>t: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -32922,7 +32864,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH61" t="inlineStr"/>
       <c r="AI61" t="inlineStr">
         <is>
           <t>trust_ethics, data_infra</t>
@@ -32933,7 +32874,6 @@
           <t>t: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -33087,14 +33027,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH62" t="inlineStr"/>
-      <c r="AI62" t="inlineStr"/>
       <c r="AJ62" t="inlineStr">
         <is>
           <t>q3: 0 -&gt; 1; q6: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -33248,7 +33185,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH63" t="inlineStr"/>
       <c r="AI63" t="inlineStr">
         <is>
           <t>integration, cognition, resources, dynamism</t>
@@ -33259,7 +33195,6 @@
           <t>q2: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -33413,7 +33348,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH64" t="inlineStr"/>
       <c r="AI64" t="inlineStr">
         <is>
           <t>dynamism, integration</t>
@@ -33424,7 +33358,6 @@
           <t>z: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -33578,7 +33511,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH65" t="inlineStr"/>
       <c r="AI65" t="inlineStr">
         <is>
           <t>trust_ethics</t>
@@ -33589,7 +33521,6 @@
           <t>q2: 1 -&gt; 0; q4: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -33743,7 +33674,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH66" t="inlineStr"/>
       <c r="AI66" t="inlineStr">
         <is>
           <t>integration, data_infra, trust_ethics, cognition</t>
@@ -33754,7 +33684,6 @@
           <t>outcome: CA -&gt; SCA; p1: c -&gt; +; t: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -33923,7 +33852,6 @@
           <t>p2: + -&gt; na; z: True -&gt; False; t: True -&gt; False; q3: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -34077,7 +34005,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH68" t="inlineStr"/>
       <c r="AI68" t="inlineStr">
         <is>
           <t>trust_ethics</t>
@@ -34088,7 +34015,6 @@
           <t>p1: + -&gt; na; s: False -&gt; True; z: False -&gt; True; t: False -&gt; True; q3: 0 -&gt; 1; q4: 0 -&gt; 1; q6: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -34242,7 +34168,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH69" t="inlineStr"/>
       <c r="AI69" t="inlineStr">
         <is>
           <t>integration</t>
@@ -34253,7 +34178,6 @@
           <t>outcome: OTHER -&gt; FP; p2: na -&gt; +; z: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -34407,7 +34331,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH70" t="inlineStr"/>
       <c r="AI70" t="inlineStr">
         <is>
           <t>dynamism</t>
@@ -34418,7 +34341,6 @@
           <t>p2: na -&gt; +</t>
         </is>
       </c>
-      <c r="AK70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -34572,7 +34494,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH71" t="inlineStr"/>
       <c r="AI71" t="inlineStr">
         <is>
           <t>trust_ethics, data_infra, integration</t>
@@ -34583,7 +34504,6 @@
           <t>s: False -&gt; True; z: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -34737,7 +34657,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH72" t="inlineStr"/>
       <c r="AI72" t="inlineStr">
         <is>
           <t>integration</t>
@@ -34748,7 +34667,6 @@
           <t>design: Qualitative/case -&gt; Mixed; outcome: OTHER -&gt; FP; s: False -&gt; True; t: False -&gt; True; q3: 0 -&gt; 1; q6: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -34902,7 +34820,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH73" t="inlineStr"/>
       <c r="AI73" t="inlineStr">
         <is>
           <t>integration, trust_ethics</t>
@@ -34913,7 +34830,6 @@
           <t>z: False -&gt; True; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -35067,7 +34983,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH74" t="inlineStr"/>
       <c r="AI74" t="inlineStr">
         <is>
           <t>integration, data_infra</t>
@@ -35078,7 +34993,6 @@
           <t>s: False -&gt; True; t: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -35232,7 +35146,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH75" t="inlineStr"/>
       <c r="AI75" t="inlineStr">
         <is>
           <t>cognition, dynamism</t>
@@ -35243,7 +35156,6 @@
           <t>p2: + -&gt; na; t: False -&gt; True; q2: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -35398,7 +35310,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH76" t="inlineStr"/>
       <c r="AI76" t="inlineStr">
         <is>
           <t>integration, platform</t>
@@ -35409,7 +35320,6 @@
           <t>tier: Core -&gt; Supporting; design: Conceptual -&gt; Survey; outcome: CA -&gt; OTHER; p1: + -&gt; na; q4: 0 -&gt; 1; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -35563,7 +35473,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH77" t="inlineStr"/>
       <c r="AI77" t="inlineStr">
         <is>
           <t>cognition</t>
@@ -35574,7 +35483,6 @@
           <t>outcome: OTHER -&gt; FP; z: True -&gt; False; t: True -&gt; False; q4: 1 -&gt; 0; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -35728,7 +35636,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH78" t="inlineStr"/>
       <c r="AI78" t="inlineStr">
         <is>
           <t>cognition, dynamism</t>
@@ -35739,7 +35646,6 @@
           <t>z: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -35908,7 +35814,6 @@
           <t>p2: + -&gt; na</t>
         </is>
       </c>
-      <c r="AK79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -36062,7 +35967,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH80" t="inlineStr"/>
       <c r="AI80" t="inlineStr">
         <is>
           <t>integration, data_infra</t>
@@ -36073,7 +35977,6 @@
           <t>p2: na -&gt; +; s: False -&gt; True; z: False -&gt; True; t: False -&gt; True; q6: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -36227,7 +36130,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH81" t="inlineStr"/>
       <c r="AI81" t="inlineStr">
         <is>
           <t>integration</t>
@@ -36238,7 +36140,6 @@
           <t>s: False -&gt; True; z: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -36392,14 +36293,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH82" t="inlineStr"/>
       <c r="AI82" t="inlineStr">
         <is>
           <t>cognition, resources</t>
         </is>
       </c>
-      <c r="AJ82" t="inlineStr"/>
-      <c r="AK82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -36564,7 +36462,6 @@
           <t>outcome: OTHER -&gt; FP; q5: 1 -&gt; 0; q6: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -36718,14 +36615,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH84" t="inlineStr"/>
       <c r="AI84" t="inlineStr">
         <is>
           <t>dynamism</t>
         </is>
       </c>
-      <c r="AJ84" t="inlineStr"/>
-      <c r="AK84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -36894,7 +36788,6 @@
           <t>p1: + -&gt; c; p2: + -&gt; na; s: False -&gt; True; t: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -37059,7 +36952,6 @@
           <t>s: True -&gt; False; q4: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -37228,7 +37120,6 @@
           <t>s: False -&gt; True; t: False -&gt; True; q2: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -37382,7 +37273,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH88" t="inlineStr"/>
       <c r="AI88" t="inlineStr">
         <is>
           <t>cognition, data_infra, dynamism</t>
@@ -37393,7 +37283,6 @@
           <t>p2: + -&gt; na; q6: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -37562,7 +37451,6 @@
           <t>q6: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -37716,14 +37604,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH90" t="inlineStr"/>
       <c r="AI90" t="inlineStr">
         <is>
           <t>integration</t>
         </is>
       </c>
-      <c r="AJ90" t="inlineStr"/>
-      <c r="AK90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -37833,7 +37718,7 @@
       </c>
       <c r="V91" s="2" t="inlineStr">
         <is>
-          <t>Abstract only; limitations not assessable unless stated in abstract</t>
+          <t>Discussion, p. 179: 'reliance on self-reported data and the focus on a single national context'</t>
         </is>
       </c>
       <c r="W91" s="2" t="n">
@@ -37856,7 +37741,7 @@
       </c>
       <c r="AC91" s="2" t="inlineStr">
         <is>
-          <t>not assessable</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AD91" s="2" t="n">
@@ -37874,10 +37759,14 @@
       </c>
       <c r="AG91" t="inlineStr">
         <is>
-          <t>Abstract-based</t>
-        </is>
-      </c>
-      <c r="AH91" t="inlineStr"/>
+          <t>Full text verified</t>
+        </is>
+      </c>
+      <c r="AH91" t="inlineStr">
+        <is>
+          <t>https://www.businessperspectives.org/images/pdf/applications/publishing/templates/article/assets/20585/IM_2024_03_Awad.pdf (published version, CC BY 4.0)</t>
+        </is>
+      </c>
       <c r="AI91" t="inlineStr">
         <is>
           <t>integration</t>
@@ -37888,7 +37777,11 @@
           <t>z: False -&gt; True; q5: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK91" t="inlineStr"/>
+      <c r="AK91" t="inlineStr">
+        <is>
+          <t>Full-text check: q7: not_assessable -&gt; yes. Full text confirms abstract coding. Direct AI-&gt;marketing innovation beta=.49 and partial mediation via organisational culture (Table 15). Culture is not a dynamic capability under the codebook, so P2 stays na. No theory named (q2=0).</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -38057,7 +37950,6 @@
           <t>design: Qualitative/case -&gt; Mixed; p2: na -&gt; +; s: False -&gt; True; z: False -&gt; True; t: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -38222,7 +38114,6 @@
           <t>design: Conceptual -&gt; Qualitative/case; s: False -&gt; True; z: False -&gt; True; t: True -&gt; False; q1: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -38292,47 +38183,47 @@
       </c>
       <c r="N94" s="2" t="inlineStr">
         <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="P94" s="2" t="inlineStr">
+        <is>
+          <t>AI contributes to supply chain resilience in five areas</t>
+        </is>
+      </c>
+      <c r="Q94" s="2" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O94" s="2" t="inlineStr">
-        <is>
-          <t>Resilience</t>
-        </is>
-      </c>
-      <c r="P94" s="2" t="inlineStr">
-        <is>
-          <t>AI contributes to supply chain resilience in five areas</t>
-        </is>
-      </c>
-      <c r="Q94" s="2" t="inlineStr">
+      <c r="R94" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="R94" s="2" t="inlineStr">
+      <c r="S94" s="2" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="T94" s="2" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="U94" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="S94" s="2" t="inlineStr">
-        <is>
-          <t>na</t>
-        </is>
-      </c>
-      <c r="T94" s="2" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="U94" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="V94" s="2" t="inlineStr">
         <is>
-          <t>Abstract only; limitations not assessable unless stated in abstract</t>
+          <t>Section 7.3 'Limitations and scope for future research' (AAM p. 32): small number of respondents, region-specific</t>
         </is>
       </c>
       <c r="W94" s="2" t="n">
@@ -38355,7 +38246,7 @@
       </c>
       <c r="AC94" s="2" t="inlineStr">
         <is>
-          <t>not assessable</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AD94" s="2" t="n">
@@ -38373,10 +38264,14 @@
       </c>
       <c r="AG94" t="inlineStr">
         <is>
-          <t>Abstract-based</t>
-        </is>
-      </c>
-      <c r="AH94" t="inlineStr"/>
+          <t>Full text verified</t>
+        </is>
+      </c>
+      <c r="AH94" t="inlineStr">
+        <is>
+          <t>https://researchonline.ljmu.ac.uk/id/eprint/15291/ (author accepted manuscript)</t>
+        </is>
+      </c>
       <c r="AI94" t="inlineStr">
         <is>
           <t>dynamism</t>
@@ -38387,7 +38282,11 @@
           <t>q2: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK94" t="inlineStr"/>
+      <c r="AK94" t="inlineStr">
+        <is>
+          <t>Full-text check: t: False -&gt; True; q7: not_assessable -&gt; yes. DC lens explicit (Sec. 4). T added: AI-enabled resilience requires 'reconfiguration of resources' framed as dynamic capability (AAM p. 26; P2/P5). P1 stays na (outcome RES).</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -38541,14 +38440,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH95" t="inlineStr"/>
-      <c r="AI95" t="inlineStr"/>
       <c r="AJ95" t="inlineStr">
         <is>
           <t>q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -38702,7 +38598,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH96" t="inlineStr"/>
       <c r="AI96" t="inlineStr">
         <is>
           <t>dynamism</t>
@@ -38713,7 +38608,6 @@
           <t>s: True -&gt; False; z: True -&gt; False; t: True -&gt; False; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -38867,7 +38761,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH97" t="inlineStr"/>
       <c r="AI97" t="inlineStr">
         <is>
           <t>integration, imitability, cognition</t>
@@ -38878,7 +38771,6 @@
           <t>z: False -&gt; True; q4: 1 -&gt; 0; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -39032,14 +38924,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH98" t="inlineStr"/>
-      <c r="AI98" t="inlineStr"/>
       <c r="AJ98" t="inlineStr">
         <is>
           <t>s: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -39193,7 +39082,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH99" t="inlineStr"/>
       <c r="AI99" t="inlineStr">
         <is>
           <t>resources, trust_ethics</t>
@@ -39362,7 +39250,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH100" t="inlineStr"/>
       <c r="AI100" t="inlineStr">
         <is>
           <t>integration, data_infra, dynamism</t>
@@ -39373,7 +39260,6 @@
           <t>s: False -&gt; True; t: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -39527,7 +39413,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH101" t="inlineStr"/>
       <c r="AI101" t="inlineStr">
         <is>
           <t>cognition</t>
@@ -39538,7 +39423,6 @@
           <t>s: True -&gt; False; z: True -&gt; False; q4: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -39707,7 +39591,6 @@
           <t>design: Survey -&gt; Mixed; p2: + -&gt; na; z: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -39861,7 +39744,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH103" t="inlineStr"/>
       <c r="AI103" t="inlineStr">
         <is>
           <t>integration, data_infra</t>
@@ -39872,7 +39754,6 @@
           <t>q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -40026,7 +39907,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH104" t="inlineStr"/>
       <c r="AI104" t="inlineStr">
         <is>
           <t>integration</t>
@@ -40037,7 +39917,6 @@
           <t>p2: + -&gt; c; q4: 1 -&gt; 0; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -40191,14 +40070,11 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH105" t="inlineStr"/>
-      <c r="AI105" t="inlineStr"/>
       <c r="AJ105" t="inlineStr">
         <is>
           <t>q4: 1 -&gt; 0; q5: 1 -&gt; 0</t>
         </is>
       </c>
-      <c r="AK105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -40352,7 +40228,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH106" t="inlineStr"/>
       <c r="AI106" t="inlineStr">
         <is>
           <t>trust_ethics, resources</t>
@@ -40363,7 +40238,6 @@
           <t>s: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -40517,7 +40391,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH107" t="inlineStr"/>
       <c r="AI107" t="inlineStr">
         <is>
           <t>resources</t>
@@ -40528,7 +40401,6 @@
           <t>p1: c -&gt; na; z: True -&gt; False</t>
         </is>
       </c>
-      <c r="AK107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -40682,7 +40554,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH108" t="inlineStr"/>
       <c r="AI108" t="inlineStr">
         <is>
           <t>platform</t>
@@ -40693,7 +40564,6 @@
           <t>p1: + -&gt; c</t>
         </is>
       </c>
-      <c r="AK108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -40803,7 +40673,7 @@
       </c>
       <c r="V109" s="2" t="inlineStr">
         <is>
-          <t>Abstract only; limitations not assessable unless stated in abstract</t>
+          <t>No limitations section; Discussion only offers future research (positive/negative data network effects, competitive advantage)</t>
         </is>
       </c>
       <c r="W109" s="2" t="n">
@@ -40826,7 +40696,7 @@
       </c>
       <c r="AC109" s="2" t="inlineStr">
         <is>
-          <t>not assessable</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AD109" s="2" t="n">
@@ -40844,10 +40714,14 @@
       </c>
       <c r="AG109" t="inlineStr">
         <is>
-          <t>Abstract-based</t>
-        </is>
-      </c>
-      <c r="AH109" t="inlineStr"/>
+          <t>Full text verified</t>
+        </is>
+      </c>
+      <c r="AH109" t="inlineStr">
+        <is>
+          <t>https://wrap.warwick.ac.uk/134220/ (author accepted manuscript, AMR)</t>
+        </is>
+      </c>
       <c r="AI109" t="inlineStr">
         <is>
           <t>platform, trust_ethics</t>
@@ -40858,7 +40732,11 @@
           <t>p1: + -&gt; na; q4: 0 -&gt; 1</t>
         </is>
       </c>
-      <c r="AK109" t="inlineStr"/>
+      <c r="AK109" t="inlineStr">
+        <is>
+          <t>Full-text check: q7: not_assessable -&gt; no. Full text confirms abstract coding: outcome perceived user value (OTHER), no DC framing, competitive advantage only named as future research.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -41012,7 +40890,6 @@
           <t>Abstract-based</t>
         </is>
       </c>
-      <c r="AH110" t="inlineStr"/>
       <c r="AI110" t="inlineStr">
         <is>
           <t>imitability, integration</t>
@@ -41023,7 +40900,6 @@
           <t>outcome: CA -&gt; SCA; s: False -&gt; True</t>
         </is>
       </c>
-      <c r="AK110" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AE110"/>
@@ -45261,12 +45137,12 @@
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>not_assessable</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Full text</t>
         </is>
       </c>
     </row>
@@ -54035,7 +53911,7 @@
       </c>
       <c r="AU53" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Full text</t>
         </is>
       </c>
     </row>
@@ -55175,7 +55051,7 @@
       </c>
       <c r="AL58" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="AM58" t="inlineStr">
@@ -55215,12 +55091,12 @@
       </c>
       <c r="AT58" t="inlineStr">
         <is>
-          <t>not_assessable</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AU58" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Full text</t>
         </is>
       </c>
     </row>
@@ -55649,12 +55525,12 @@
       </c>
       <c r="AL60" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="AM60" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="AN60" t="inlineStr">
@@ -55694,7 +55570,7 @@
       </c>
       <c r="AU60" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Full text</t>
         </is>
       </c>
     </row>
@@ -56365,7 +56241,7 @@
       </c>
       <c r="AM63" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="AN63" t="inlineStr">
@@ -56390,7 +56266,7 @@
       </c>
       <c r="AR63" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AS63" t="inlineStr">
@@ -56400,12 +56276,12 @@
       </c>
       <c r="AT63" t="inlineStr">
         <is>
-          <t>not_assessable</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AU63" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Full text</t>
         </is>
       </c>
     </row>
@@ -58992,12 +58868,12 @@
       </c>
       <c r="AQ74" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AR74" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AS74" t="inlineStr">
@@ -59007,12 +58883,12 @@
       </c>
       <c r="AT74" t="inlineStr">
         <is>
-          <t>not_assessable</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AU74" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Full text</t>
         </is>
       </c>
     </row>
@@ -66828,12 +66704,12 @@
       </c>
       <c r="AT107" t="inlineStr">
         <is>
-          <t>not_assessable</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AU107" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Full text</t>
         </is>
       </c>
     </row>
@@ -67504,7 +67380,7 @@
       </c>
       <c r="AM110" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="AN110" t="inlineStr">
@@ -67539,15 +67415,16 @@
       </c>
       <c r="AT110" t="inlineStr">
         <is>
-          <t>not_assessable</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="AU110" t="inlineStr">
         <is>
-          <t>Abstract</t>
-        </is>
-      </c>
-    </row>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="111"/>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>

</xml_diff>